<commit_message>
feat: Mark final round yellow warnings as completed (Dashboard)
</commit_message>
<xml_diff>
--- a/SgsNextschool/backend/WP16_งานค้าง_ต้นทาง.xlsx
+++ b/SgsNextschool/backend/WP16_งานค้าง_ต้นทาง.xlsx
@@ -6580,7 +6580,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>2026-09-30 20:26:37</t>
+          <t>Wed Sep 30 2026 20:26:37 GMT+0700 (เวลาอินโดจีน)</t>
         </is>
       </c>
     </row>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>2026-09-30 20:26:37</t>
+          <t>Wed Sep 30 2026 20:26:37 GMT+0700 (เวลาอินโดจีน)</t>
         </is>
       </c>
     </row>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>2026-09-30 20:26:37</t>
+          <t>Wed Sep 30 2026 20:26:37 GMT+0700 (เวลาอินโดจีน)</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8824,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>2026-09-30 20:26:37</t>
+          <t>Wed Sep 30 2026 20:26:37 GMT+0700 (เวลาอินโดจีน)</t>
         </is>
       </c>
     </row>
@@ -11748,7 +11748,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>2026-09-30 20:26:37</t>
+          <t>Wed Sep 30 2026 20:26:37 GMT+0700 (เวลาอินโดจีน)</t>
         </is>
       </c>
     </row>

</xml_diff>